<commit_message>
Show the year and RM on their own row in ledgers and journals
Ledger accounts now use Date | Particulars | Folio | Amount with the
year on the first row under the headings and RM in the Amount column.
Entries show only the month and day, and a new year row starts when
the year changes. Journals follow the same pattern with RM under Debit
and Credit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cg2FRYV2NgKh9WWDoLcpR2
</commit_message>
<xml_diff>
--- a/excel/Ch12_Accounting_Concepts.xlsx
+++ b/excel/Ch12_Accounting_Concepts.xlsx
@@ -96,10 +96,10 @@
     <t xml:space="preserve">Formats used</t>
   </si>
   <si>
-    <t xml:space="preserve">Journal: Date | Particulars | Debit (RM) | Credit (RM).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ledger account: Dr side and Cr side, each with Date | Particulars | Folio | Amount (RM). Folio: GJ = general journal, CB = cash book.</t>
+    <t xml:space="preserve">Journal: Date | Particulars | Debit | Credit. The first row shows the year, with RM under Debit and Credit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ledger account: Dr side and Cr side, each with Date | Particulars | Folio | Amount. The first row under the headings shows the year, with RM in the Amount column; entries then show the month and day. Folio: GJ = general journal, CB = cash book.</t>
   </si>
   <si>
     <t xml:space="preserve">Statement of Profit or Loss: marker (Add / Less) | Particulars | RM | RM | RM.</t>
@@ -1798,7 +1798,7 @@
       <c r="AE19" s="4"/>
       <c r="AF19" s="4"/>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
         <v>16</v>
       </c>

</xml_diff>